<commit_message>
style: rename Grade 4 attachment folders to align with P4list.txt
- Renamed 9 folder names under the '\''四年級'\'' directory to establish 100% exact character matches with '\''P4list.txt'\''.

- Added '\''P4list.txt'\'' tracking list to the repository.
</commit_message>
<xml_diff>
--- a/履歷表 6A31黃熹澄/附件/四年級/四年級 附件 清單_.xlsx
+++ b/履歷表 6A31黃熹澄/附件/四年級/四年級 附件 清單_.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="file_checking_report" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="P4" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,180 +12,288 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="135">
+  <si>
+    <t xml:space="preserve">STEAM </t>
+  </si>
+  <si>
+    <t>2025 FIRST LEGO League Asia Open Championship The Third Place</t>
+  </si>
   <si>
     <t>編號 (No.)</t>
   </si>
   <si>
+    <t>First Lego league 香港錦標賽 2024至2025 overall second runner-up</t>
+  </si>
+  <si>
+    <t>First Lego league 香港錦標賽 2024至2025 Team model award</t>
+  </si>
+  <si>
     <t>文件夾名稱 (Folder Name)</t>
   </si>
   <si>
+    <t>2024-2025全港校際 STEAM 資優盃資訊科技 總決賽學霸第一名</t>
+  </si>
+  <si>
     <t>檔案名稱 (File Name)</t>
   </si>
   <si>
+    <t>WSC certificate of competition Asia Pacific challenge silver award</t>
+  </si>
+  <si>
     <t>狀態 (Status)</t>
   </si>
   <si>
+    <t>Innovation and technology excellence with marty the robot AT BETT 2025</t>
+  </si>
+  <si>
     <t>2024年參加迦密柏雨中學舉辦之科學達人大挑戰參與證明</t>
   </si>
   <si>
+    <t>大埔公立學校2024至2025學年度代表香港到境外交流獎學金</t>
+  </si>
+  <si>
     <t>2024年參加迦密柏雨中學舉辦之科學達人大挑戰參與證明.pdf</t>
   </si>
   <si>
+    <t>Best presentation award at the second global Marty challenge</t>
+  </si>
+  <si>
     <t>MATCH</t>
   </si>
   <si>
+    <t>Robofest Hong Kong RoboParade Junior 2025 Gold  Award</t>
+  </si>
+  <si>
     <t>2024至2025全港校際Steam資優盃資訊科技初賽金獎</t>
   </si>
   <si>
     <t>2024至2025全港校際Steam資優盃資訊科技初賽金獎.pdf</t>
   </si>
   <si>
+    <t>Robofest Hong Kong BottleSumo 2025 Junior Gold Award</t>
+  </si>
+  <si>
     <t>2024至2025學年參加Sport ACT獎勵計劃並獲金獎</t>
   </si>
   <si>
+    <t>大埔舊墟公立學校2024至2025學年度科學科技獎勵計劃獎學金</t>
+  </si>
+  <si>
     <t>2024至2025學年參加Sport ACT獎勵計劃並獲金獎.pdf</t>
   </si>
   <si>
+    <t>香港電腦教育學會 資訊科技挑戰獎勵計劃 銀章級</t>
+  </si>
+  <si>
     <t>AI assisted film virtual production</t>
   </si>
   <si>
     <t>AI assisted film virtual production.pdf</t>
   </si>
   <si>
+    <t>AI Assisted Film Virtual Production</t>
+  </si>
+  <si>
+    <t>NOW TV STEM AWARDS Silver</t>
+  </si>
+  <si>
     <t>AI singer unleashed Potentials</t>
   </si>
   <si>
     <t>AI singer unleashed Potentials.pdf</t>
   </si>
   <si>
-    <t>Best presentation award at the second global Marty challenge</t>
+    <t>香港機械人學院 2024-2025學年度下學期機 械人精英培訓課程 表現優良</t>
+  </si>
+  <si>
+    <t>小學聯合校steam比賽2025 參加證明</t>
   </si>
   <si>
     <t>Best presentation award at the second global Marty challenge.pdf</t>
   </si>
   <si>
+    <t>迦密柏雨中學 舉辦之科學達人大挑戰 2024 參與證明</t>
+  </si>
+  <si>
     <t>First Lego league 香港錦標賽二四至二五overall second runner-up</t>
   </si>
   <si>
     <t>First Lego league 香港錦標賽二四至二五overall second runner-up.pdf</t>
   </si>
   <si>
+    <t>Global Classroom class of 2025 certificate of participation</t>
+  </si>
+  <si>
     <t>First Lego league香港錦標賽2024至2025 Team model award</t>
   </si>
   <si>
+    <t>體育</t>
+  </si>
+  <si>
     <t>First Lego league香港錦標賽2024至2025 Team model award.pdf</t>
   </si>
   <si>
-    <t>Global Classroom class of 2025 certificate of participation</t>
+    <t>第九屆協恩中學聯合小學籃球邀請賽參與證書</t>
   </si>
   <si>
     <t>Global Classroom class of 2025 certificate of participation.pdf</t>
   </si>
   <si>
+    <t>國學證書參加武藝操學習</t>
+  </si>
+  <si>
     <t>Hong Kong School Elite Competition 2025 English group P4 Bronze award</t>
   </si>
   <si>
     <t>Hong Kong School Elite Competition 2025 English group P4 Bronze award.pdf</t>
   </si>
   <si>
+    <t>「躍動校園活力人生」邁步巴黎奧運挑戰賽暨MVPA60金章</t>
+  </si>
+  <si>
     <t>Hong Kong schools music and speech association 76th Hong Kong school speech festival 2024 solo verse speaking non-open primary for girls second place</t>
   </si>
   <si>
     <t>Hong Kong schools music and speech association 76th Hong Kong school speech festival 2024 solo verse speaking non-open primary for girls second place.pdf</t>
   </si>
   <si>
-    <t>Innovation and technology excellence with marty the robot AT BETT 2025</t>
+    <t>林大輝中學全港小學籃球邀請賽參與證書</t>
   </si>
   <si>
     <t>Innovation and technology excellence with marty the robot AT BETT 2025.pdf</t>
   </si>
   <si>
+    <t>視覺藝術</t>
+  </si>
+  <si>
+    <t>AI Singer | Elderly &amp; Youth Together Unleashed Potentials</t>
+  </si>
+  <si>
     <t>Now TV stem獎勵計劃silver</t>
   </si>
   <si>
     <t>Now TV stem獎勵計劃silver.pdf</t>
   </si>
   <si>
+    <t>香港光雕節 參與證書</t>
+  </si>
+  <si>
     <t>Robofast Hong Kong RoboParade gold award 2024</t>
   </si>
   <si>
     <t>Robofast Hong Kong RoboParade gold award 2024.pdf</t>
   </si>
   <si>
+    <t>第一屆非遺旗袍設計比賽入圍獎</t>
+  </si>
+  <si>
     <t>Robofast Hong Kong roboContest Silver award 2024</t>
   </si>
   <si>
+    <t>青少年兒童當代繪畫大賽2025 金獎</t>
+  </si>
+  <si>
     <t>Robofast Hong Kong roboContest Silver award 2024.pdf</t>
   </si>
   <si>
     <t>Robofest  Hong Kong roboParade Junior Gold  award</t>
   </si>
   <si>
+    <t>香港拔萃兒童文化藝術協會certificate of achievement</t>
+  </si>
+  <si>
     <t>Robofest  Hong Kong roboParade Junior Gold  award.pdf</t>
   </si>
   <si>
     <t>Robofest Hong Kong junior bottleSumo gold award 2025</t>
   </si>
   <si>
+    <t>大埔舊墟公立學校「愛的創意校園」視覺創科成果展AI虛擬歌手獎</t>
+  </si>
+  <si>
     <t>Robofest Hong Kong junior bottleSumo gold award 2025.pdf</t>
   </si>
   <si>
+    <t>大埔舊墟公立學校 2024至2025學年度傑出藝術成就獎</t>
+  </si>
+  <si>
     <t>S PC少兒普通話水平測試等級證書A等</t>
   </si>
   <si>
     <t>S PC少兒普通話水平測試等級證書A等.pdf</t>
   </si>
   <si>
-    <t>WSC certificate of competition Asia Pacific challenge silver award</t>
+    <t>大埔舊墟公立學校「愛的創意校園視藝創科成果展」優秀作品獎</t>
+  </si>
+  <si>
+    <t>大埔舊墟公立學校大埔舊墟公立學校家長教師會2024至2025學年親子環保生活用品設計比賽高小組銀獎</t>
   </si>
   <si>
     <t>WSC certificate of competition Asia Pacific challenge silver award.pdf</t>
   </si>
   <si>
-    <t>「躍動校園活力人生」邁步巴黎奧運挑戰賽暨MVPA60金章</t>
+    <t>第13屆世界兒童繪畫大獎賽2024優秀獎</t>
   </si>
   <si>
     <t>「躍動校園活力人生」邁步巴黎奧運挑戰賽暨MVPA60金章.pdf</t>
   </si>
   <si>
+    <t>大埔警區 防騙許願寶牒設計比賽 高小組 亞軍</t>
+  </si>
+  <si>
     <t>中國香港學界體育聯會2024至2025年度大埔區小學校際籃球比賽季軍</t>
   </si>
   <si>
     <t>中國香港學界體育聯會2024至2025年度大埔區小學校際籃球比賽季軍.pdf</t>
   </si>
   <si>
-    <t>國學證書參加武藝操學習</t>
+    <t>朗誦</t>
   </si>
   <si>
     <t>國學證書參加武藝操學習.pdf</t>
   </si>
   <si>
-    <t>大埔公立學校2024至2025學年度代表香港到境外交流獎學金</t>
+    <t>Hong Kong Schools Music and Speech Association 76th Hong Kong School Speech Festival 2024 Solo Verse Speaking Non-Open primary 4 Girls Second Place</t>
   </si>
   <si>
     <t>大埔公立學校2024至2025學年度代表香港到境外交流獎學金.pdf</t>
   </si>
   <si>
+    <t>SPC少兒普通話水平測試等級證書A等</t>
+  </si>
+  <si>
     <t>大埔區學生獎勵計劃2024至2025表現優異</t>
   </si>
   <si>
     <t>大埔區學生獎勵計劃2024至2025表現優異.pdf</t>
   </si>
   <si>
-    <t>大埔舊墟公立學校 2024至2025學年度傑出藝術成就獎</t>
+    <t>香港學校音樂及朗誦協會 第76屆 香港學校朗誦戰2024 散文獨誦粵語四年級女子組 季軍</t>
+  </si>
+  <si>
+    <t>音樂</t>
   </si>
   <si>
     <t>大埔舊墟公立學校 2024至2025學年度傑出藝術成就獎.pdf</t>
   </si>
   <si>
+    <t>第22屆全港小學英文文國組合歌唱比賽榮獲分組優異獎</t>
+  </si>
+  <si>
+    <t>第22屆英文民歌歌唱比賽初賽 舊墟之聲 小學組 分組冠軍</t>
+  </si>
+  <si>
     <t>大埔舊墟公立學校2024至2025學年度學業成績榮譽獎</t>
   </si>
   <si>
     <t>大埔舊墟公立學校2024至2025學年度學業成績榮譽獎.pdf</t>
   </si>
   <si>
-    <t>大埔舊墟公立學校2024至2025學年度科學科技獎勵計劃獎學金</t>
+    <t>第22屆英文民歌歌唱比賽決賽 舊墟之聲 小學組 最佳動作演繹獎、優異獎、全場殿軍</t>
+  </si>
+  <si>
+    <t>領袖、校內與社會服務</t>
   </si>
   <si>
     <t>大埔舊墟公立學校2024至2025學年度科學科技獎勵計劃獎學金.pdf</t>
@@ -193,42 +302,48 @@
     <t>大埔舊墟公立學校2024至2025學年道擔任風紀表現優異記優點一次</t>
   </si>
   <si>
+    <t>教育局公益少年團大埔委員會小學中級獎章證書</t>
+  </si>
+  <si>
     <t>大埔舊墟公立學校2024至2025學年道擔任風紀表現優異記優點一次.pdf</t>
   </si>
   <si>
+    <t>大埔警區大埔區提子大使委任狀</t>
+  </si>
+  <si>
     <t>大埔舊墟公立學校2024至2025學年閱讀獎勵計劃銅獎</t>
   </si>
   <si>
     <t>大埔舊墟公立學校2024至2025學年閱讀獎勵計劃銅獎.pdf</t>
   </si>
   <si>
-    <t>大埔舊墟公立學校「愛的創意校園」視覺創科成果展AI虛擬歌手獎</t>
+    <t>大埔警區提子大使2024至2025年度感謝狀</t>
   </si>
   <si>
     <t>大埔舊墟公立學校「愛的創意校園」視覺創科成果展AI虛擬歌手獎.pdf</t>
   </si>
   <si>
-    <t>大埔舊墟公立學校「愛的創意校園視藝創科成果展」優秀作品獎</t>
+    <t>大埔舊墟公立學校2024至2025學年度 學業成績榮譽獎</t>
   </si>
   <si>
     <t>大埔舊墟公立學校「愛的創意校園視藝創科成果展」優秀作品獎.pdf</t>
   </si>
   <si>
-    <t>大埔舊墟公立學校大埔舊墟公立學校家長教師會2024至2025學年親子環保生活用品設計比賽高小組銀獎</t>
+    <t>大埔舊墟公立學校2024至2025學年度 擔任風紀表現優異記優點一次</t>
   </si>
   <si>
     <t>大埔舊墟公立學校大埔舊墟公立學校家長教師會2024至2025學年親子環保生活用品設計比賽高小組銀獎.pdf</t>
   </si>
   <si>
-    <t>大埔警區大埔區提子大使委任狀</t>
+    <t>大埔舊墟公立學校2024至2025學年 閱讀獎勵計劃銅獎</t>
+  </si>
+  <si>
+    <t>舊墟學校好孩子獎勵計劃完成本獎勵計劃優異四星章</t>
   </si>
   <si>
     <t>大埔警區大埔區提子大使委任狀.pdf</t>
   </si>
   <si>
-    <t>大埔警區提子大使2024至2025年度感謝狀</t>
-  </si>
-  <si>
     <t>大埔警區提子大使2024至2025年度感謝狀.pdf</t>
   </si>
   <si>
@@ -238,27 +353,15 @@
     <t>小學聯合校steam比賽2025參加證明.pdf</t>
   </si>
   <si>
-    <t>教育局公益少年團大埔委員會小學中級獎章證書</t>
-  </si>
-  <si>
     <t>教育局公益少年團大埔委員會小學中級獎章證書.pdf</t>
   </si>
   <si>
-    <t>林大輝中學全港小學籃球邀請賽參與證書</t>
-  </si>
-  <si>
     <t>林大輝中學全港小學籃球邀請賽參與證書.pdf</t>
   </si>
   <si>
-    <t>第13屆世界兒童繪畫大獎賽2024優秀獎</t>
-  </si>
-  <si>
     <t>第13屆世界兒童繪畫大獎賽2024優秀獎.pdf</t>
   </si>
   <si>
-    <t>第22屆全港小學英文文國組合歌唱比賽榮獲分組優異獎</t>
-  </si>
-  <si>
     <t>第22屆全港小學英文文國組合歌唱比賽榮獲分組優異獎.pdf</t>
   </si>
   <si>
@@ -274,21 +377,12 @@
     <t>第22屆英文民國歌唱比賽決賽舊墟之聲榮獲小學組最佳動作演繹獎、優異獎、全場殿軍.pdf</t>
   </si>
   <si>
-    <t>第一屆非遺旗袍設計比賽入圍獎</t>
-  </si>
-  <si>
     <t>第一屆非遺旗袍設計比賽入圍獎.pdf</t>
   </si>
   <si>
-    <t>第九屆協恩中學聯合小學籃球邀請賽參與證書</t>
-  </si>
-  <si>
     <t>第九屆協恩中學聯合小學籃球邀請賽參與證書.pdf</t>
   </si>
   <si>
-    <t>舊墟學校好孩子獎勵計劃完成本獎勵計劃優異四星章</t>
-  </si>
-  <si>
     <t>舊墟學校好孩子獎勵計劃完成本獎勵計劃優異四星章.pdf</t>
   </si>
   <si>
@@ -298,9 +392,6 @@
     <t>資訊科技挑戰獎勵計劃銀章級.pdf</t>
   </si>
   <si>
-    <t>青少年兒童當代繪畫大賽2025 金獎</t>
-  </si>
-  <si>
     <t>青少年兒童當代繪畫大賽2025 金獎.pdf</t>
   </si>
   <si>
@@ -317,9 +408,6 @@
   </si>
   <si>
     <t>香港學校音樂及朗誦協會第76屆香港學校朗誦戰2024散文獨誦粵語四年級女子組季軍.pdf</t>
-  </si>
-  <si>
-    <t>香港拔萃兒童文化藝術協會certificate of achievement</t>
   </si>
   <si>
     <t>香港拔萃兒童文化藝術協會certificate of achievement.pdf</t>
@@ -378,6 +466,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -586,33 +678,34 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="20.63"/>
     <col customWidth="1" min="2" max="2" width="130.88"/>
     <col customWidth="1" min="3" max="3" width="119.88"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -620,13 +713,13 @@
         <v>1.0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -634,13 +727,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +741,13 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -662,13 +755,13 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -676,13 +769,13 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -690,13 +783,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -704,24 +797,24 @@
         <v>9.0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +822,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -743,13 +836,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -757,13 +850,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -771,13 +864,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -785,13 +878,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
@@ -799,13 +892,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -813,13 +906,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -827,13 +920,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
@@ -841,13 +934,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -855,13 +948,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -869,13 +962,13 @@
         <v>20.0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -883,13 +976,13 @@
         <v>21.0</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
@@ -897,13 +990,13 @@
         <v>22.0</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24">
@@ -911,13 +1004,13 @@
         <v>23.0</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
@@ -925,13 +1018,13 @@
         <v>24.0</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26">
@@ -939,13 +1032,13 @@
         <v>25.0</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27">
@@ -953,13 +1046,13 @@
         <v>26.0</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28">
@@ -967,13 +1060,13 @@
         <v>27.0</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29">
@@ -981,13 +1074,13 @@
         <v>28.0</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30">
@@ -995,13 +1088,13 @@
         <v>29.0</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>61</v>
+        <v>99</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -1009,13 +1102,13 @@
         <v>30.0</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
@@ -1023,13 +1116,13 @@
         <v>31.0</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>66</v>
+        <v>104</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">
@@ -1037,13 +1130,13 @@
         <v>32.0</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -1051,13 +1144,13 @@
         <v>33.0</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>70</v>
+        <v>109</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35">
@@ -1065,13 +1158,13 @@
         <v>34.0</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>72</v>
+        <v>110</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36">
@@ -1079,13 +1172,13 @@
         <v>35.0</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
@@ -1093,13 +1186,13 @@
         <v>36.0</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38">
@@ -1107,13 +1200,13 @@
         <v>37.0</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39">
@@ -1121,13 +1214,13 @@
         <v>38.0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40">
@@ -1135,13 +1228,13 @@
         <v>39.0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41">
@@ -1149,13 +1242,13 @@
         <v>40.0</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42">
@@ -1163,13 +1256,13 @@
         <v>41.0</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43">
@@ -1177,13 +1270,13 @@
         <v>42.0</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44">
@@ -1191,13 +1284,13 @@
         <v>43.0</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45">
@@ -1205,13 +1298,13 @@
         <v>44.0</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46">
@@ -1219,13 +1312,13 @@
         <v>45.0</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47">
@@ -1233,13 +1326,13 @@
         <v>46.0</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48">
@@ -1247,13 +1340,13 @@
         <v>47.0</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
     </row>
     <row r="49">
@@ -1261,13 +1354,13 @@
         <v>48.0</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50">
@@ -1275,13 +1368,13 @@
         <v>49.0</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51">
@@ -1289,13 +1382,439 @@
         <v>50.0</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>104</v>
+        <v>133</v>
       </c>
       <c r="C51" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="32.25"/>
+    <col customWidth="1" min="2" max="2" width="120.88"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="1">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="1">
+        <v>11.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="1">
+        <v>12.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="1">
+        <v>13.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="1">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1">
+        <v>15.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1">
+        <v>16.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="1">
+        <v>17.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="1">
+        <v>18.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="1">
+        <v>19.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="1">
+        <v>20.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="1">
+        <v>21.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="1">
+        <v>22.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="1">
+        <v>23.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="1">
+        <v>24.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="1">
+        <v>25.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="1">
+        <v>26.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="1">
+        <v>27.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="1">
+        <v>28.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="1">
+        <v>29.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="1">
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="1">
+        <v>31.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1">
+        <v>32.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="1">
+        <v>33.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="1">
+        <v>34.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="1">
+        <v>35.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C36" s="1">
+        <v>36.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C37" s="1">
+        <v>37.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C38" s="1">
+        <v>38.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" s="1">
+        <v>39.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" s="1">
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="1">
+        <v>41.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" s="1">
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C43" s="1">
+        <v>43.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C44" s="1">
+        <v>44.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C45" s="1">
+        <v>45.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" s="1">
+        <v>46.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D51" s="1" t="s">
-        <v>6</v>
+      <c r="C47" s="1">
+        <v>47.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C48" s="1">
+        <v>48.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C49" s="1">
+        <v>49.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>